<commit_message>
Campus services: doctor timings, one tuck & food tab, rep links
Medical opens on the doctor's week, with no numbers of its own, then
the medical unit, ambulance, gynecologist, pharmacies, psychologist and
psychiatrist.

Shops and Food are one tab, "Tuck Shops and Food" (the tab reads "Tuck
& Food" so four fit on a 360px phone; the heading gives the full name).
Delivery shows whether a shop delivers, not what it charges: the menu
screen works out the fee for the student's own place. Kotler Da does
not deliver.

The hostel tabs drop the reps and night messes, which have screens of
their own. A "Contact the OH Rep" row now links to POR details, searched
down to that one rep, instead of carrying a copy of the number; back
returns to the same hostel tab. LVH's "rep or LVH admin" reads "LVH Rep"
through CORRECTIONS, since there is no admin contact to give.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Campus Contacts.template.xlsx
+++ b/templates/Campus Contacts.template.xlsx
@@ -484,16 +484,8 @@
           <t>Doctor</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>9876543211</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>9876543212</t>
-        </is>
-      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>